<commit_message>
Corrigir importação para permitir múltiplas matrículas e exibir todos alunos na aba Todos
- Modificada lógica de importação para permitir múltiplas matrículas para o mesmo aluno
- Verificação de duplicata agora considera nome + telefone + professor + curso
- Alunos com múltiplos cursos podem ser importados corretamente
- Aba 'Todos' de pagamentos agora exibe todos os alunos matriculados com seus status
- Corrigida indentação no código de pagamentos
</commit_message>
<xml_diff>
--- a/exemplo_importacao_alunos.xlsx
+++ b/exemplo_importacao_alunos.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="193">
   <si>
     <t xml:space="preserve">nome</t>
   </si>
@@ -148,7 +148,16 @@
     <t xml:space="preserve">29/03/2025</t>
   </si>
   <si>
-    <t xml:space="preserve">PERIC</t>
+    <t xml:space="preserve">Gabriel PERIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 96074-0877</t>
+  </si>
+  <si>
+    <t xml:space="preserve">São Paulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP</t>
   </si>
   <si>
     <t xml:space="preserve">03/04/2025</t>
@@ -157,18 +166,39 @@
     <t xml:space="preserve">Quinta-feira</t>
   </si>
   <si>
+    <t xml:space="preserve">19:00 às 21:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">Matheus Moreski</t>
   </si>
   <si>
+    <t xml:space="preserve">65 9356-2063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MT</t>
+  </si>
+  <si>
     <t xml:space="preserve">mãe Fernanda </t>
   </si>
   <si>
     <t xml:space="preserve">MARK</t>
   </si>
   <si>
+    <t xml:space="preserve">21 99929-0869</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio de Janeiro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RJ</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sábado</t>
   </si>
   <si>
+    <t xml:space="preserve">10:00 às 12:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">ERICK JENUINO DEBIAZI</t>
   </si>
   <si>
@@ -184,6 +214,12 @@
     <t xml:space="preserve">BRUNA AUEBACH</t>
   </si>
   <si>
+    <t xml:space="preserve">47 9763-5094</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC</t>
+  </si>
+  <si>
     <t xml:space="preserve">03/07/2025</t>
   </si>
   <si>
@@ -202,6 +238,9 @@
     <t xml:space="preserve">Jacqueline Mendes Magalhães</t>
   </si>
   <si>
+    <t xml:space="preserve">21 99367-1641</t>
+  </si>
+  <si>
     <t xml:space="preserve">18/07/2025</t>
   </si>
   <si>
@@ -211,18 +250,21 @@
     <t xml:space="preserve">21 98986-1122</t>
   </si>
   <si>
-    <t xml:space="preserve">Rio de Janeiro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RJ</t>
-  </si>
-  <si>
     <t xml:space="preserve">20/09/2025</t>
   </si>
   <si>
     <t xml:space="preserve">GABRIEL SANCHES SERQUEIRA</t>
   </si>
   <si>
+    <t xml:space="preserve">61 433 429 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brasília</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DF</t>
+  </si>
+  <si>
     <t xml:space="preserve">20/08/2025</t>
   </si>
   <si>
@@ -241,9 +283,6 @@
     <t xml:space="preserve">19 98170-3566</t>
   </si>
   <si>
-    <t xml:space="preserve">SP</t>
-  </si>
-  <si>
     <t xml:space="preserve">01/10/2025</t>
   </si>
   <si>
@@ -253,9 +292,6 @@
     <t xml:space="preserve">47 9707-5558</t>
   </si>
   <si>
-    <t xml:space="preserve">SC</t>
-  </si>
-  <si>
     <t xml:space="preserve">17/10/2025</t>
   </si>
   <si>
@@ -307,6 +343,9 @@
     <t xml:space="preserve">31/05/2025</t>
   </si>
   <si>
+    <t xml:space="preserve">10:30 às 12:30</t>
+  </si>
+  <si>
     <t xml:space="preserve">PAULO ROBERTO SANTOS DA SILVA</t>
   </si>
   <si>
@@ -343,7 +382,7 @@
     <t xml:space="preserve">25/09/2025</t>
   </si>
   <si>
-    <t xml:space="preserve">EXPERIMENTAL Gabriella dos Santos</t>
+    <t xml:space="preserve">Gabriella dos Santos</t>
   </si>
   <si>
     <t xml:space="preserve">00000-0000</t>
@@ -382,6 +421,9 @@
     <t xml:space="preserve">17/05/2025</t>
   </si>
   <si>
+    <t xml:space="preserve">09:00 às 11:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">PEDRO LUCAS BARRETO </t>
   </si>
   <si>
@@ -415,9 +457,6 @@
     <t xml:space="preserve">11 95648-5992</t>
   </si>
   <si>
-    <t xml:space="preserve">São Paulo</t>
-  </si>
-  <si>
     <t xml:space="preserve">Niveo Diegues</t>
   </si>
   <si>
@@ -427,6 +466,9 @@
     <t xml:space="preserve">Quarta-feira</t>
   </si>
   <si>
+    <t xml:space="preserve">19:30 às 22:30</t>
+  </si>
+  <si>
     <t xml:space="preserve">LETÍCIA ALVES OLIVEIRA </t>
   </si>
   <si>
@@ -445,6 +487,9 @@
     <t xml:space="preserve">26/07/2025</t>
   </si>
   <si>
+    <t xml:space="preserve">09:30 às 11:30</t>
+  </si>
+  <si>
     <t xml:space="preserve">DAVI ARENA LEAL</t>
   </si>
   <si>
@@ -478,6 +523,9 @@
     <t xml:space="preserve">27/08/2025</t>
   </si>
   <si>
+    <t xml:space="preserve">15:00 às 18:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">LARISSA GERONIMO</t>
   </si>
   <si>
@@ -487,6 +535,9 @@
     <t xml:space="preserve">Sorocaba</t>
   </si>
   <si>
+    <t xml:space="preserve">10:00 às 13:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">MARINA CARREGOSA RODRIGUES</t>
   </si>
   <si>
@@ -520,6 +571,9 @@
     <t xml:space="preserve">Cecília Carvalho</t>
   </si>
   <si>
+    <t xml:space="preserve">14:30 às 16:30</t>
+  </si>
+  <si>
     <t xml:space="preserve">Guilherme de Figueiredo Rimola</t>
   </si>
   <si>
@@ -533,6 +587,9 @@
   </si>
   <si>
     <t xml:space="preserve">20/07/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:00 às 20:00</t>
   </si>
   <si>
     <t xml:space="preserve">PEDRO SUCUPIRA </t>
@@ -558,6 +615,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -580,6 +638,7 @@
       <color rgb="FFFFFFFF"/>
       <name val="Cambria"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -981,7 +1040,15 @@
       <c r="A4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>45</v>
+      </c>
       <c r="E4" s="0" t="s">
         <v>29</v>
       </c>
@@ -995,7 +1062,7 @@
         <v>31</v>
       </c>
       <c r="L4" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M4" s="0" t="s">
         <v>31</v>
@@ -1004,7 +1071,7 @@
         <v>31</v>
       </c>
       <c r="O4" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P4" s="0" t="s">
         <v>31</v>
@@ -1022,24 +1089,34 @@
         <v>33</v>
       </c>
       <c r="U4" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V4" s="2" t="n">
         <v>300</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="X4" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y4" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="4"/>
+        <v>49</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>51</v>
+      </c>
       <c r="E5" s="0" t="s">
         <v>29</v>
       </c>
@@ -1047,7 +1124,7 @@
         <v>5</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="J5" s="0" t="s">
         <v>31</v>
@@ -1056,7 +1133,7 @@
         <v>31</v>
       </c>
       <c r="L5" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M5" s="0" t="s">
         <v>31</v>
@@ -1065,7 +1142,7 @@
         <v>31</v>
       </c>
       <c r="O5" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P5" s="0" t="s">
         <v>31</v>
@@ -1083,24 +1160,34 @@
         <v>33</v>
       </c>
       <c r="U5" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V5" s="2" t="n">
         <v>300</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="X5" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y5" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="4"/>
+        <v>53</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>56</v>
+      </c>
       <c r="E6" s="0" t="s">
         <v>29</v>
       </c>
@@ -1114,7 +1201,7 @@
         <v>31</v>
       </c>
       <c r="L6" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M6" s="0" t="s">
         <v>31</v>
@@ -1123,7 +1210,7 @@
         <v>31</v>
       </c>
       <c r="O6" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P6" s="0" t="s">
         <v>31</v>
@@ -1148,22 +1235,24 @@
       </c>
       <c r="W6" s="4"/>
       <c r="X6" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y6" s="2"/>
+        <v>57</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>29</v>
@@ -1179,7 +1268,7 @@
         <v>31</v>
       </c>
       <c r="L7" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M7" s="0" t="s">
         <v>31</v>
@@ -1188,7 +1277,7 @@
         <v>31</v>
       </c>
       <c r="O7" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P7" s="0" t="s">
         <v>31</v>
@@ -1206,24 +1295,34 @@
         <v>33</v>
       </c>
       <c r="U7" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V7" s="2" t="n">
         <v>350</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="X7" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y7" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" s="4"/>
+        <v>63</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>65</v>
+      </c>
       <c r="E8" s="0" t="s">
         <v>29</v>
       </c>
@@ -1237,16 +1336,16 @@
         <v>31</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M8" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N8" s="0" t="s">
         <v>31</v>
       </c>
       <c r="O8" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P8" s="0" t="s">
         <v>31</v>
@@ -1264,25 +1363,27 @@
         <v>33</v>
       </c>
       <c r="U8" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V8" s="2" t="n">
         <v>300</v>
       </c>
       <c r="W8" s="3" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="X8" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y8" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>28</v>
@@ -1306,7 +1407,7 @@
         <v>31</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N9" s="0" t="s">
         <v>31</v>
@@ -1330,24 +1431,34 @@
         <v>33</v>
       </c>
       <c r="U9" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V9" s="2" t="n">
         <v>280</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="X9" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>70</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="4"/>
+        <v>71</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>56</v>
+      </c>
       <c r="E10" s="0" t="s">
         <v>29</v>
       </c>
@@ -1394,25 +1505,27 @@
         <v>300</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="X10" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y10" s="2"/>
+        <v>57</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E11" s="0" t="s">
         <v>29</v>
@@ -1427,7 +1540,7 @@
         <v>31</v>
       </c>
       <c r="L11" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M11" s="0" t="s">
         <v>31</v>
@@ -1436,7 +1549,7 @@
         <v>31</v>
       </c>
       <c r="O11" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P11" s="0" t="s">
         <v>31</v>
@@ -1460,18 +1573,28 @@
         <v>260</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="X11" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>57</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="4"/>
+        <v>77</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>80</v>
+      </c>
       <c r="E12" s="0" t="s">
         <v>29</v>
       </c>
@@ -1486,7 +1609,7 @@
         <v>31</v>
       </c>
       <c r="L12" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M12" s="0" t="s">
         <v>31</v>
@@ -1495,7 +1618,7 @@
         <v>31</v>
       </c>
       <c r="O12" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P12" s="0" t="s">
         <v>31</v>
@@ -1513,31 +1636,33 @@
         <v>33</v>
       </c>
       <c r="U12" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V12" s="2" t="n">
         <v>300</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="X12" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>70</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E13" s="0" t="s">
         <v>29</v>
@@ -1552,7 +1677,7 @@
         <v>31</v>
       </c>
       <c r="L13" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M13" s="0" t="s">
         <v>31</v>
@@ -1561,7 +1686,7 @@
         <v>31</v>
       </c>
       <c r="O13" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P13" s="0" t="s">
         <v>31</v>
@@ -1579,31 +1704,33 @@
         <v>33</v>
       </c>
       <c r="U13" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V13" s="2" t="n">
         <v>260</v>
       </c>
       <c r="W13" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="X13" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="X13" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y13" s="2"/>
+      <c r="Y13" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E14" s="0" t="s">
         <v>29</v>
@@ -1619,7 +1746,7 @@
         <v>31</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M14" s="0" t="s">
         <v>31</v>
@@ -1628,7 +1755,7 @@
         <v>31</v>
       </c>
       <c r="O14" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P14" s="0" t="s">
         <v>31</v>
@@ -1637,7 +1764,7 @@
         <v>32</v>
       </c>
       <c r="R14" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S14" s="0" t="s">
         <v>31</v>
@@ -1646,30 +1773,33 @@
         <v>33</v>
       </c>
       <c r="U14" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V14" s="2" t="n">
         <v>340</v>
       </c>
       <c r="W14" s="3" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="X14" s="0" t="s">
-        <v>58</v>
+        <v>70</v>
+      </c>
+      <c r="Y14" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E15" s="0" t="s">
         <v>29</v>
@@ -1684,7 +1814,7 @@
         <v>31</v>
       </c>
       <c r="L15" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M15" s="0" t="s">
         <v>31</v>
@@ -1693,7 +1823,7 @@
         <v>31</v>
       </c>
       <c r="O15" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P15" s="0" t="s">
         <v>31</v>
@@ -1711,30 +1841,33 @@
         <v>33</v>
       </c>
       <c r="U15" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V15" s="2" t="n">
         <v>340</v>
       </c>
       <c r="W15" s="3" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="X15" s="0" t="s">
-        <v>58</v>
+        <v>70</v>
+      </c>
+      <c r="Y15" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="E16" s="0" t="s">
         <v>29</v>
@@ -1749,7 +1882,7 @@
         <v>31</v>
       </c>
       <c r="L16" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M16" s="0" t="s">
         <v>31</v>
@@ -1758,7 +1891,7 @@
         <v>31</v>
       </c>
       <c r="O16" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P16" s="0" t="s">
         <v>31</v>
@@ -1776,30 +1909,33 @@
         <v>33</v>
       </c>
       <c r="U16" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V16" s="2" t="n">
         <v>300</v>
       </c>
       <c r="W16" s="3" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="X16" s="0" t="s">
-        <v>58</v>
+        <v>70</v>
+      </c>
+      <c r="Y16" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E17" s="0" t="s">
         <v>29</v>
@@ -1814,7 +1950,7 @@
         <v>31</v>
       </c>
       <c r="L17" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M17" s="0" t="s">
         <v>31</v>
@@ -1823,7 +1959,7 @@
         <v>31</v>
       </c>
       <c r="O17" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P17" s="0" t="s">
         <v>31</v>
@@ -1832,7 +1968,7 @@
         <v>32</v>
       </c>
       <c r="R17" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S17" s="0" t="s">
         <v>31</v>
@@ -1841,31 +1977,33 @@
         <v>33</v>
       </c>
       <c r="U17" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V17" s="2" t="n">
         <v>300</v>
       </c>
       <c r="W17" s="3" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="X17" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y17" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="E18" s="0" t="s">
         <v>29</v>
@@ -1880,7 +2018,7 @@
         <v>31</v>
       </c>
       <c r="L18" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M18" s="0" t="s">
         <v>31</v>
@@ -1889,7 +2027,7 @@
         <v>31</v>
       </c>
       <c r="O18" s="0" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P18" s="0" t="s">
         <v>31</v>
@@ -1907,30 +2045,33 @@
         <v>33</v>
       </c>
       <c r="U18" s="0" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V18" s="2" t="n">
         <v>280</v>
       </c>
       <c r="W18" s="3" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="X18" s="0" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+      <c r="Y18" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E19" s="0" t="s">
         <v>29</v>
@@ -1969,7 +2110,7 @@
         <v>31</v>
       </c>
       <c r="T19" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="U19" s="0" t="s">
         <v>12</v>
@@ -1978,24 +2119,27 @@
         <v>360</v>
       </c>
       <c r="W19" s="3" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="X19" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y19" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E20" s="0" t="s">
         <v>29</v>
@@ -2034,7 +2178,7 @@
         <v>31</v>
       </c>
       <c r="T20" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="U20" s="0" t="s">
         <v>12</v>
@@ -2043,24 +2187,27 @@
         <v>260</v>
       </c>
       <c r="W20" s="3" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="X20" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y20" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E21" s="0" t="s">
         <v>29</v>
@@ -2099,7 +2246,7 @@
         <v>31</v>
       </c>
       <c r="T21" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="U21" s="0" t="s">
         <v>12</v>
@@ -2108,24 +2255,27 @@
         <v>280</v>
       </c>
       <c r="W21" s="3" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="X21" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y21" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E22" s="0" t="s">
         <v>29</v>
@@ -2164,7 +2314,7 @@
         <v>31</v>
       </c>
       <c r="T22" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="U22" s="0" t="s">
         <v>12</v>
@@ -2173,24 +2323,27 @@
         <v>280</v>
       </c>
       <c r="W22" s="3" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="X22" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y22" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E23" s="0" t="s">
         <v>29</v>
@@ -2229,7 +2382,7 @@
         <v>31</v>
       </c>
       <c r="T23" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="U23" s="0" t="s">
         <v>12</v>
@@ -2238,18 +2391,21 @@
         <v>300</v>
       </c>
       <c r="W23" s="3" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="X23" s="0" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>57</v>
+      </c>
+      <c r="Y23" s="0" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="E24" s="0" t="s">
         <v>29</v>
@@ -2286,7 +2442,7 @@
         <v>32</v>
       </c>
       <c r="T24" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="U24" s="0" t="s">
         <v>12</v>
@@ -2295,24 +2451,27 @@
         <v>60</v>
       </c>
       <c r="W24" s="3" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="X24" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y24" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E25" s="0" t="s">
         <v>29</v>
@@ -2351,7 +2510,7 @@
         <v>31</v>
       </c>
       <c r="T25" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="U25" s="0" t="s">
         <v>12</v>
@@ -2360,24 +2519,27 @@
         <v>280</v>
       </c>
       <c r="W25" s="3" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="X25" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y25" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E26" s="0" t="s">
         <v>29</v>
@@ -2416,7 +2578,7 @@
         <v>31</v>
       </c>
       <c r="T26" s="0" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="U26" s="0" t="s">
         <v>12</v>
@@ -2425,24 +2587,27 @@
         <v>280</v>
       </c>
       <c r="W26" s="3" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="X26" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y26" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E27" s="0" t="s">
         <v>29</v>
@@ -2481,7 +2646,7 @@
         <v>31</v>
       </c>
       <c r="T27" s="0" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="U27" s="0" t="s">
         <v>12</v>
@@ -2490,24 +2655,27 @@
         <v>260</v>
       </c>
       <c r="W27" s="3" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="X27" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y27" s="0" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E28" s="0" t="s">
         <v>29</v>
@@ -2546,7 +2714,7 @@
         <v>31</v>
       </c>
       <c r="T28" s="0" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="U28" s="0" t="s">
         <v>12</v>
@@ -2555,24 +2723,27 @@
         <v>340</v>
       </c>
       <c r="W28" s="3" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="X28" s="0" t="s">
-        <v>123</v>
+        <v>137</v>
+      </c>
+      <c r="Y28" s="0" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E29" s="0" t="s">
         <v>29</v>
@@ -2581,10 +2752,10 @@
         <v>15</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="J29" s="0" t="s">
         <v>31</v>
@@ -2617,7 +2788,7 @@
         <v>31</v>
       </c>
       <c r="T29" s="0" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="U29" s="0" t="s">
         <v>12</v>
@@ -2626,15 +2797,18 @@
         <v>600</v>
       </c>
       <c r="W29" s="3" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="X29" s="0" t="s">
-        <v>123</v>
+        <v>137</v>
+      </c>
+      <c r="Y29" s="0" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B30" s="4"/>
       <c r="E30" s="0" t="s">
@@ -2674,7 +2848,7 @@
         <v>31</v>
       </c>
       <c r="T30" s="0" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="U30" s="0" t="s">
         <v>12</v>
@@ -2683,21 +2857,21 @@
         <v>290</v>
       </c>
       <c r="W30" s="3" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E31" s="0" t="s">
         <v>29</v>
@@ -2736,7 +2910,7 @@
         <v>31</v>
       </c>
       <c r="T31" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U31" s="0" t="s">
         <v>12</v>
@@ -2745,24 +2919,27 @@
         <v>360</v>
       </c>
       <c r="W31" s="3" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="X31" s="0" t="s">
-        <v>134</v>
+        <v>147</v>
+      </c>
+      <c r="Y31" s="0" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E32" s="0" t="s">
         <v>29</v>
@@ -2801,7 +2978,7 @@
         <v>31</v>
       </c>
       <c r="T32" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U32" s="0" t="s">
         <v>12</v>
@@ -2810,24 +2987,27 @@
         <v>360</v>
       </c>
       <c r="W32" s="3" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="X32" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
+      </c>
+      <c r="Y32" s="0" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E33" s="0" t="s">
         <v>29</v>
@@ -2866,7 +3046,7 @@
         <v>31</v>
       </c>
       <c r="T33" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U33" s="0" t="s">
         <v>12</v>
@@ -2875,24 +3055,27 @@
         <v>400</v>
       </c>
       <c r="W33" s="3" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="X33" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y33" s="0" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E34" s="0" t="s">
         <v>29</v>
@@ -2931,7 +3114,7 @@
         <v>31</v>
       </c>
       <c r="T34" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U34" s="0" t="s">
         <v>12</v>
@@ -2940,24 +3123,27 @@
         <v>360</v>
       </c>
       <c r="W34" s="3" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="X34" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y34" s="0" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E35" s="0" t="s">
         <v>29</v>
@@ -2996,7 +3182,7 @@
         <v>31</v>
       </c>
       <c r="T35" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U35" s="0" t="s">
         <v>12</v>
@@ -3005,24 +3191,27 @@
         <v>380</v>
       </c>
       <c r="W35" s="3" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="X35" s="0" t="s">
-        <v>134</v>
+        <v>147</v>
+      </c>
+      <c r="Y35" s="0" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E36" s="0" t="s">
         <v>29</v>
@@ -3061,7 +3250,7 @@
         <v>31</v>
       </c>
       <c r="T36" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U36" s="0" t="s">
         <v>12</v>
@@ -3070,24 +3259,27 @@
         <v>400</v>
       </c>
       <c r="W36" s="3" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="X36" s="0" t="s">
-        <v>134</v>
+        <v>147</v>
+      </c>
+      <c r="Y36" s="0" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>149</v>
+        <v>164</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E37" s="0" t="s">
         <v>29</v>
@@ -3126,7 +3318,7 @@
         <v>31</v>
       </c>
       <c r="T37" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U37" s="0" t="s">
         <v>12</v>
@@ -3135,24 +3327,27 @@
         <v>400</v>
       </c>
       <c r="W37" s="3" t="s">
-        <v>151</v>
+        <v>166</v>
       </c>
       <c r="X37" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y37" s="0" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E38" s="0" t="s">
         <v>29</v>
@@ -3191,7 +3386,7 @@
         <v>31</v>
       </c>
       <c r="T38" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U38" s="0" t="s">
         <v>12</v>
@@ -3200,24 +3395,27 @@
         <v>310</v>
       </c>
       <c r="W38" s="3" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="X38" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y38" s="0" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E39" s="0" t="s">
         <v>29</v>
@@ -3256,7 +3454,7 @@
         <v>31</v>
       </c>
       <c r="T39" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U39" s="0" t="s">
         <v>12</v>
@@ -3265,24 +3463,27 @@
         <v>360</v>
       </c>
       <c r="W39" s="3" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="X39" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y39" s="0" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E40" s="0" t="s">
         <v>29</v>
@@ -3319,7 +3520,7 @@
         <v>31</v>
       </c>
       <c r="T40" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U40" s="0" t="s">
         <v>12</v>
@@ -3328,22 +3529,25 @@
         <v>360</v>
       </c>
       <c r="W40" s="3" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="X40" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y40" s="0" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E41" s="0" t="s">
         <v>29</v>
@@ -3380,7 +3584,7 @@
         <v>31</v>
       </c>
       <c r="T41" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U41" s="0" t="s">
         <v>12</v>
@@ -3389,24 +3593,24 @@
         <v>380</v>
       </c>
       <c r="W41" s="3" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="X41" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E42" s="0" t="s">
         <v>29</v>
@@ -3442,7 +3646,7 @@
         <v>31</v>
       </c>
       <c r="T42" s="0" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="U42" s="0" t="s">
         <v>12</v>
@@ -3451,24 +3655,27 @@
         <v>400</v>
       </c>
       <c r="W42" s="3" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="X42" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y42" s="0" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E43" s="0" t="s">
         <v>29</v>
@@ -3507,7 +3714,7 @@
         <v>31</v>
       </c>
       <c r="T43" s="0" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="U43" s="0" t="s">
         <v>12</v>
@@ -3516,21 +3723,24 @@
         <v>280</v>
       </c>
       <c r="X43" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y43" s="0" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E44" s="0" t="s">
         <v>29</v>
@@ -3569,7 +3779,7 @@
         <v>31</v>
       </c>
       <c r="T44" s="0" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="U44" s="0" t="s">
         <v>12</v>
@@ -3578,22 +3788,27 @@
         <v>350</v>
       </c>
       <c r="W44" s="3" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="X44" s="0" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="Y44" s="0" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B45" s="4"/>
+        <v>74</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="C45" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E45" s="0" t="s">
         <v>29</v>
@@ -3632,7 +3847,7 @@
         <v>31</v>
       </c>
       <c r="T45" s="0" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="U45" s="0" t="s">
         <v>12</v>
@@ -3641,24 +3856,27 @@
         <v>300</v>
       </c>
       <c r="W45" s="3" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="X45" s="0" t="s">
-        <v>134</v>
+        <v>147</v>
+      </c>
+      <c r="Y45" s="0" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E46" s="0" t="s">
         <v>29</v>
@@ -3693,8 +3911,11 @@
       <c r="R46" s="0" t="s">
         <v>32</v>
       </c>
+      <c r="S46" s="0" t="s">
+        <v>31</v>
+      </c>
       <c r="T46" s="0" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="U46" s="0" t="s">
         <v>12</v>
@@ -3703,10 +3924,13 @@
         <v>300</v>
       </c>
       <c r="W46" s="3" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="X46" s="0" t="s">
-        <v>134</v>
+        <v>147</v>
+      </c>
+      <c r="Y46" s="0" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrigir timezone de datas e atualizar gráfico de evolução para usar data de início
- Corrigido problema de timezone: backend agora retorna datas no formato YYYY-MM-DD (sem timestamp)
- Função formatDate atualizada para tratar strings ISO com ou sem timestamp
- Gráfico de Evolução de Alunos agora considera data_inicio da matrícula ao invés de data_cadastro
- Atualizada descrição do gráfico para refletir que usa data de início
</commit_message>
<xml_diff>
--- a/exemplo_importacao_alunos.xlsx
+++ b/exemplo_importacao_alunos.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="198">
   <si>
     <t xml:space="preserve">nome</t>
   </si>
@@ -385,7 +385,10 @@
     <t xml:space="preserve">Gabriella dos Santos</t>
   </si>
   <si>
-    <t xml:space="preserve">00000-0000</t>
+    <t xml:space="preserve">99 12345-6789</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A</t>
   </si>
   <si>
     <t xml:space="preserve">01/11/2025</t>
@@ -451,6 +454,9 @@
     <t xml:space="preserve">GABRIEL BARBOSA</t>
   </si>
   <si>
+    <t xml:space="preserve">21 97121-1726</t>
+  </si>
+  <si>
     <t xml:space="preserve">ALTANIS LOURENÇO </t>
   </si>
   <si>
@@ -554,6 +560,15 @@
   </si>
   <si>
     <t xml:space="preserve">GIOVANE MATHEUS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 98556-1166</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vanessa Mãe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 99231-6969</t>
   </si>
   <si>
     <t xml:space="preserve">DEBORA OLIVEIRA DA SILVA</t>
@@ -2407,6 +2422,12 @@
       <c r="B24" s="2" t="s">
         <v>121</v>
       </c>
+      <c r="C24" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" s="0" t="s">
+        <v>122</v>
+      </c>
       <c r="E24" s="0" t="s">
         <v>29</v>
       </c>
@@ -2451,7 +2472,7 @@
         <v>60</v>
       </c>
       <c r="W24" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="X24" s="0" t="s">
         <v>57</v>
@@ -2462,10 +2483,10 @@
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C25" s="0" t="s">
         <v>55</v>
@@ -2519,7 +2540,7 @@
         <v>280</v>
       </c>
       <c r="W25" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="X25" s="0" t="s">
         <v>57</v>
@@ -2530,10 +2551,10 @@
     </row>
     <row r="26" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C26" s="0" t="s">
         <v>55</v>
@@ -2587,7 +2608,7 @@
         <v>280</v>
       </c>
       <c r="W26" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="X26" s="0" t="s">
         <v>57</v>
@@ -2598,10 +2619,10 @@
     </row>
     <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C27" s="0" t="s">
         <v>55</v>
@@ -2646,7 +2667,7 @@
         <v>31</v>
       </c>
       <c r="T27" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="U27" s="0" t="s">
         <v>12</v>
@@ -2655,21 +2676,21 @@
         <v>260</v>
       </c>
       <c r="W27" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="X27" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y27" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C28" s="0" t="s">
         <v>55</v>
@@ -2714,7 +2735,7 @@
         <v>31</v>
       </c>
       <c r="T28" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="U28" s="0" t="s">
         <v>12</v>
@@ -2723,10 +2744,10 @@
         <v>340</v>
       </c>
       <c r="W28" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="X28" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Y28" s="0" t="s">
         <v>48</v>
@@ -2734,10 +2755,10 @@
     </row>
     <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C29" s="0" t="s">
         <v>55</v>
@@ -2752,11 +2773,11 @@
         <v>15</v>
       </c>
       <c r="G29" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="H29" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="H29" s="0" t="s">
-        <v>139</v>
-      </c>
       <c r="J29" s="0" t="s">
         <v>31</v>
       </c>
@@ -2788,7 +2809,7 @@
         <v>31</v>
       </c>
       <c r="T29" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="U29" s="0" t="s">
         <v>12</v>
@@ -2797,10 +2818,10 @@
         <v>600</v>
       </c>
       <c r="W29" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="X29" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Y29" s="0" t="s">
         <v>48</v>
@@ -2808,9 +2829,17 @@
     </row>
     <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="B30" s="4"/>
+        <v>143</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>56</v>
+      </c>
       <c r="E30" s="0" t="s">
         <v>29</v>
       </c>
@@ -2848,7 +2877,7 @@
         <v>31</v>
       </c>
       <c r="T30" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="U30" s="0" t="s">
         <v>12</v>
@@ -2857,15 +2886,15 @@
         <v>290</v>
       </c>
       <c r="W30" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C31" s="0" t="s">
         <v>44</v>
@@ -2910,7 +2939,7 @@
         <v>31</v>
       </c>
       <c r="T31" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U31" s="0" t="s">
         <v>12</v>
@@ -2919,21 +2948,21 @@
         <v>360</v>
       </c>
       <c r="W31" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="X31" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Y31" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C32" s="0" t="s">
         <v>44</v>
@@ -2978,7 +3007,7 @@
         <v>31</v>
       </c>
       <c r="T32" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U32" s="0" t="s">
         <v>12</v>
@@ -2987,21 +3016,21 @@
         <v>360</v>
       </c>
       <c r="W32" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="X32" s="0" t="s">
         <v>47</v>
       </c>
       <c r="Y32" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C33" s="0" t="s">
         <v>44</v>
@@ -3046,7 +3075,7 @@
         <v>31</v>
       </c>
       <c r="T33" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U33" s="0" t="s">
         <v>12</v>
@@ -3055,21 +3084,21 @@
         <v>400</v>
       </c>
       <c r="W33" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="X33" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y33" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C34" s="0" t="s">
         <v>44</v>
@@ -3114,7 +3143,7 @@
         <v>31</v>
       </c>
       <c r="T34" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U34" s="0" t="s">
         <v>12</v>
@@ -3123,21 +3152,21 @@
         <v>360</v>
       </c>
       <c r="W34" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="X34" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y34" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C35" s="0" t="s">
         <v>44</v>
@@ -3182,7 +3211,7 @@
         <v>31</v>
       </c>
       <c r="T35" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U35" s="0" t="s">
         <v>12</v>
@@ -3191,21 +3220,21 @@
         <v>380</v>
       </c>
       <c r="W35" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="X35" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Y35" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C36" s="0" t="s">
         <v>44</v>
@@ -3250,7 +3279,7 @@
         <v>31</v>
       </c>
       <c r="T36" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U36" s="0" t="s">
         <v>12</v>
@@ -3262,18 +3291,18 @@
         <v>69</v>
       </c>
       <c r="X36" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Y36" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C37" s="0" t="s">
         <v>44</v>
@@ -3318,7 +3347,7 @@
         <v>31</v>
       </c>
       <c r="T37" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U37" s="0" t="s">
         <v>12</v>
@@ -3327,24 +3356,24 @@
         <v>400</v>
       </c>
       <c r="W37" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="X37" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y37" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>45</v>
@@ -3386,7 +3415,7 @@
         <v>31</v>
       </c>
       <c r="T38" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U38" s="0" t="s">
         <v>12</v>
@@ -3395,21 +3424,21 @@
         <v>310</v>
       </c>
       <c r="W38" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="X38" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y38" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C39" s="0" t="s">
         <v>44</v>
@@ -3454,7 +3483,7 @@
         <v>31</v>
       </c>
       <c r="T39" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U39" s="0" t="s">
         <v>12</v>
@@ -3463,21 +3492,21 @@
         <v>360</v>
       </c>
       <c r="W39" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="X39" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y39" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C40" s="0" t="s">
         <v>44</v>
@@ -3520,7 +3549,7 @@
         <v>31</v>
       </c>
       <c r="T40" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U40" s="0" t="s">
         <v>12</v>
@@ -3529,20 +3558,22 @@
         <v>360</v>
       </c>
       <c r="W40" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="X40" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y40" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B41" s="4"/>
+        <v>179</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>180</v>
+      </c>
       <c r="C41" s="0" t="s">
         <v>44</v>
       </c>
@@ -3553,6 +3584,12 @@
         <v>29</v>
       </c>
       <c r="F41" s="4"/>
+      <c r="G41" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="H41" s="0" t="s">
+        <v>182</v>
+      </c>
       <c r="J41" s="0" t="s">
         <v>32</v>
       </c>
@@ -3584,7 +3621,7 @@
         <v>31</v>
       </c>
       <c r="T41" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U41" s="0" t="s">
         <v>12</v>
@@ -3593,7 +3630,7 @@
         <v>380</v>
       </c>
       <c r="W41" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="X41" s="0" t="s">
         <v>57</v>
@@ -3601,10 +3638,10 @@
     </row>
     <row r="42" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C42" s="0" t="s">
         <v>44</v>
@@ -3646,7 +3683,7 @@
         <v>31</v>
       </c>
       <c r="T42" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U42" s="0" t="s">
         <v>12</v>
@@ -3655,21 +3692,21 @@
         <v>400</v>
       </c>
       <c r="W42" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="X42" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y42" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C43" s="0" t="s">
         <v>55</v>
@@ -3714,7 +3751,7 @@
         <v>31</v>
       </c>
       <c r="T43" s="0" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="U43" s="0" t="s">
         <v>12</v>
@@ -3726,15 +3763,15 @@
         <v>57</v>
       </c>
       <c r="Y43" s="0" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C44" s="0" t="s">
         <v>55</v>
@@ -3779,7 +3816,7 @@
         <v>31</v>
       </c>
       <c r="T44" s="0" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="U44" s="0" t="s">
         <v>12</v>
@@ -3788,13 +3825,13 @@
         <v>350</v>
       </c>
       <c r="W44" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="X44" s="0" t="s">
         <v>57</v>
       </c>
       <c r="Y44" s="0" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3847,7 +3884,7 @@
         <v>31</v>
       </c>
       <c r="T45" s="0" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="U45" s="0" t="s">
         <v>12</v>
@@ -3856,21 +3893,21 @@
         <v>300</v>
       </c>
       <c r="W45" s="3" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="X45" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Y45" s="0" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C46" s="0" t="s">
         <v>55</v>
@@ -3915,7 +3952,7 @@
         <v>31</v>
       </c>
       <c r="T46" s="0" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="U46" s="0" t="s">
         <v>12</v>
@@ -3924,13 +3961,13 @@
         <v>300</v>
       </c>
       <c r="W46" s="3" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="X46" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Y46" s="0" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>